<commit_message>
doc: add evidence to module 7
</commit_message>
<xml_diff>
--- a/Tests/excel/module07_test_cases.xlsx
+++ b/Tests/excel/module07_test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test-case-academic-portal\Tests\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DA6D1D-4EB3-417A-B47D-8ECB85E3082B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C9123D-8CE4-4846-A122-5AECC3E77FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4237,7 +4237,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="95.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="147" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>246</v>
       </c>

</xml_diff>